<commit_message>
update  fallback iccid in model and others
</commit_message>
<xml_diff>
--- a/Skytronsystem/skytron_api/static/StockUpload.xlsx
+++ b/Skytronsystem/skytron_api/static/StockUpload.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THE LOGICBOX\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kisha\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92C5F81F-47D8-4D9A-B7F0-0FE9C1426D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA1D6F5-A4DA-4EA5-B05A-F9F97E9D6659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4485" yWindow="4875" windowWidth="24405" windowHeight="10590" xr2:uid="{D0AB19E0-B29D-4663-843D-2660DBE7C963}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="18432" windowHeight="10680" xr2:uid="{D0AB19E0-B29D-4663-843D-2660DBE7C963}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="28">
   <si>
     <t>123456789012</t>
   </si>
@@ -97,6 +97,18 @@
   </si>
   <si>
     <t>SlNo</t>
+  </si>
+  <si>
+    <t>iccid2</t>
+  </si>
+  <si>
+    <t>234557890123</t>
+  </si>
+  <si>
+    <t>234567893123</t>
+  </si>
+  <si>
+    <t>123456189012</t>
   </si>
 </sst>
 </file>
@@ -154,9 +166,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -194,7 +206,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -300,7 +312,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -442,7 +454,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -450,22 +462,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CA243AE-2080-4012-B02B-C735788549C2}">
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="1"/>
-    <col min="3" max="3" width="16.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" style="1" customWidth="1"/>
-    <col min="7" max="8" width="12" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13" style="1" customWidth="1"/>
-    <col min="10" max="10" width="19.5703125" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" style="1"/>
+    <col min="3" max="4" width="16.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.88671875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="18.88671875" style="1" customWidth="1"/>
+    <col min="8" max="9" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19.5546875" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>23</v>
       </c>
@@ -476,28 +488,31 @@
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -508,28 +523,31 @@
         <v>0</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="2">
+      <c r="J2" s="2">
         <v>45352</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -540,28 +558,31 @@
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I3" s="2">
+      <c r="J3" s="2">
         <v>45353</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -572,24 +593,27 @@
         <v>1</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="H4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="2">
+      <c r="J4" s="2">
         <v>45353</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>